<commit_message>
Reordena el día 5: Pokémon en Qianhai y luces al viernes.
UpperHills y el Pop Mart van primero, luego Lianhua, la tienda de la前海壹方城, CoCo Park, Harmay y Shuiwei. El espectáculo del Civic Center queda anotado para el viernes.

Co-authored-by: Arturo Real Lucas <ArturoReal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/viaje-china/dia-05-shenzhen.xlsx
+++ b/viaje-china/dia-05-shenzhen.xlsx
@@ -9,12 +9,15 @@
   <sheets>
     <sheet name="Horario" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ruta principal" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Alternativas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Viernes y alternativas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Horario'!$A$5:$C$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ruta principal'!$A$4:$J$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Alternativas'!$A$4:$I$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Horario'!$5:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ruta principal'!$A$4:$J$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ruta principal'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Viernes y alternativas'!$A$4:$H$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Viernes y alternativas'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,12 +48,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -110,16 +113,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -493,36 +496,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Día 5 — jueves 5 de noviembre de 2026 — Shenzhen (Futian)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
+          <t>Día 5 — jueves 5 de noviembre de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1 € = 7,55 ¥ (4 oct 2026), euros redondeados. La comisión de Imagine va aparte. Todas las salidas están contadas desde el hotel: 滨河大道5022号联合广场A座, metro 岗厦 salida E.</t>
+          <t>1 € = 7,55 ¥ (4 oct 2026). Hotel: 滨河大道5022号联合广场A座, metro 岗厦 salida E. Orden: UpperHills y Pop Mart, Lianhua, Pokémon en la前海壹方城, CoCo Park, Harmay, Shuiwei. Las luces del Civic Center pasan al viernes 6.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Texto para el taxi: 请到福田区滨河大道5022号联合广场A座，LuxCabins花园宾舍酒店，岗厦地铁站E口</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+          <t>Taxi del aeropuerto: 请到福田区滨河大道5022号联合广场A座，LuxCabins花园宾舍酒店，岗厦地铁站E口</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Hora</t>
@@ -539,7 +542,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="78" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>07:10</t>
@@ -556,7 +559,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="78" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>08:00–08:30</t>
@@ -564,7 +567,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Taxi oficial, puerta 13 del centro de transporte</t>
+          <t>Taxi oficial, puerta 13</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -573,7 +576,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="78" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>09:15–10:00</t>
@@ -586,19 +589,19 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>No salgáis a ver sitios con las maletas</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="78" customHeight="1">
+          <t>No salgáis con las maletas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>10:15–10:40</t>
+          <t>10:20–12:00</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Metro a UpperHills</t>
+          <t>UpperHills, Pop Mart y algo de comer</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -607,144 +610,136 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="78" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>10:40–12:30</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>UpperHills, Pop Mart y comida</t>
+          <t>Puente a Lianhua y mirador</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Se puede dejar en una hora</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="78" customHeight="1">
+          <t>Una hora basta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>12:30–14:15</t>
+          <t>13:10–14:00</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Puente a Lianhua Hill y mirador</t>
+          <t>Taxi a la前海壹方城 (Uniwalk)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>El parque sigue abierto por la tarde</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="78" customHeight="1">
+          <t>40–60 min. Texto: 请到宝安区新湖路99号前海壹方城，宝安中心地铁站F口</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>14:15–15:00</t>
+          <t>14:00–16:00</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Bajada a pie por el CBD</t>
+          <t>Centro Pokémon, planta B2, zona 捣谷岛谷</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Las luces de las torres son a las 19:00, no ahora</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="78" customHeight="1">
+          <t>Jueves 10:00–22:00. Entrada gratis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>15:00–16:30</t>
+          <t>16:10–17:00</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
+          <t>Metro línea 1 hasta CoCo Park</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Dirección 罗湖, bajada en 购物公园. Mejor que el taxi a esa hora</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>17:00–18:00</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
           <t>CoCo Park</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Se puede saltar</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="78" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>16:30–19:00</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Hotel: check-in, ducha y una hora tumbados</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>No lo quitéis</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="78" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>19:00–20:15</t>
+          <t>18:10–19:00</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>A pie hasta Harmay y Riad</t>
+          <t>Harmay, a 10 min a pie del hotel</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Riad se puede mover a otra noche en Futian</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="78" customHeight="1">
+          <t>Cierra a las 22:00. Se salta si solo queréis el Pop Mart</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>20:15–22:00</t>
+          <t>19:15–21:00</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Metro a Shuiwei, cena y vuelta al hotel</t>
+          <t>Shuiwei y vuelta al hotel</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Los puestos siguen hasta cerca de las 2:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Si salís del hotel antes de las 10:00, invertid el bloque de la mañana: primero Lianhua (abre a las 6:00) y a las 10:00 cruzad el puente a UpperHills. El resto del día no cambia.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:C16"/>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LDía 5 · 5 nov 2026 · Shenzhen Futian</oddHeader>
+    <oddHeader>&amp;LDía 5 · 5 nov 2026 · Shenzhen</oddHeader>
     <oddFooter>&amp;R1 € = 7,55 ¥ · 4 oct 2026</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -760,36 +755,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ruta principal del día 5 — desde el hotel</t>
+          <t>Ruta principal del día 5 — orden confirmado</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>El día sí se puede hacer: todo está en el corredor norte-sur de Futian. Shuiwei va el último porque abre a las 16:00. Harmay y Riad van de noche, a pie, cuando las torres se encienden (19:00–22:00). Un jueves no hace falta reserva para verlas desde la calle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>El Pokémon está en Bao'an, no en Futian. Desde Lianhua se va en taxi. La vuelta en metro línea 1 deja en CoCo Park. Pop Mart se hace dentro de UpperHills. Harmay está junto al hotel, no en UpperHills, y va antes de Shuiwei porque cierra a las 22:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Orden</t>
@@ -837,11 +832,11 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Amap (enlace corto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="78" customHeight="1">
+          <t>Amap corto</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>0</t>
@@ -854,7 +849,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Llegada 07:10. Taxis las 24 h</t>
+          <t>Llegada 07:10. Taxis 24 h</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -864,7 +859,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>No sale del hotel. Taxi oficial en la puerta 13. Mejor con maletas: 50–80 min en hora punta. Plan B: línea 11 dirección 岗厦北, bajada en 岗厦北 (unos 35 min) y 10–15 min a pie.</t>
+          <t>No sale del hotel. Taxi en la puerta 13, 50–80 min con maletas. Plan B: línea 11 dirección 岗厦北, bajada en 岗厦北, 10–15 min a pie.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -874,7 +869,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Dejáis maletas en el hotel y seguís al punto 1.</t>
+          <t>Maletas al hotel y metro al punto 1.</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -893,7 +888,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="78" customHeight="1">
+    <row r="6" ht="84" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>1</t>
@@ -906,27 +901,27 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>10:00–22:00 (viernes y sábado hasta las 22:30)</t>
+          <t>10:00–22:00</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Entrada gratis. Comida para dos en el centro: 150–300 ¥ (20–40 €)</t>
+          <t>Entrada gratis. Comida para dos 150–300 ¥ (20–40 €)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Metro, mejor opción. Línea 10 en 岗厦, dirección 双拥街, 3 paradas, 冬瓜岭, salida E, 8 min a pie. Unos 25 min, unos 4 ¥ (0,50 €) por persona. Taxi 15–25 min, 20–40 ¥ (3–5 €).</t>
+          <t>Metro. Línea 10 en 岗厦, dirección 双拥街, 3 paradas, 冬瓜岭, salida E, 8 min a pie. Unos 25 min, unos 4 ¥ por persona. Taxi 15–25 min, 20–40 ¥ (3–5 €).</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Línea 10 dirección 福田口岸 hasta 岗厦, salida E, y 5 min a pie. Taxi 15–20 min.</t>
+          <t>Línea 10 dirección 福田口岸 hasta 岗厦, salida E.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>A pie por el puente hasta Lianhua Hill, 10–20 min. No volváis al hotel.</t>
+          <t>A pie por el puente a Lianhua, 10–20 min.</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -945,7 +940,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="78" customHeight="1">
+    <row r="7" ht="84" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>1b</t>
@@ -958,27 +953,27 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>El mismo horario del centro, desde las 10:00</t>
+          <t>El mismo horario del centro</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Entrada gratis. Caja ciega habitual 59–79 ¥ (8–10 €); depende de la serie</t>
+          <t>Entrada gratis. Caja ciega habitual 59–79 ¥ (8–10 €)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>El mismo metro que UpperHills. No es otro desplazamiento.</t>
+          <t>El mismo metro que UpperHills. Se hace en esta parada, no al final del día.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>El mismo regreso que UpperHills.</t>
+          <t>El mismo regreso.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Seguid al puente hacia Lianhua sin salir del recinto.</t>
+          <t>Seguid al puente hacia Lianhua.</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -997,7 +992,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="78" customHeight="1">
+    <row r="8" ht="84" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>2</t>
@@ -1020,17 +1015,17 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Si ya estáis en UpperHills, a pie por el puente (10–20 min). Desde el hotel directo: taxi 15 min, 20–35 ¥ (3–5 €). Metro: línea 10 hasta 莲花村 y un paseo; el taxi o el puente son más simples.</t>
+          <t>Si venís de UpperHills, a pie por el puente. Desde el hotel: taxi 15 min, 20–35 ¥ (3–5 €).</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Taxi 15 min, 20–35 ¥. En metro: bajad por el sur hasta 少年宫, línea 4 hasta 会展中心 y línea 1 una parada hasta 岗厦.</t>
+          <t>Taxi 15 min. Metro: 少年宫, línea 4 a 会展中心 y línea 1 a 岗厦.</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>A pie hacia el sur, 30–40 min, por el Civic Center hasta CoCo Park.</t>
+          <t>Taxi directo a la前海壹方城. No paréis en CoCo Park de camino.</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -1049,7 +1044,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="78" customHeight="1">
+    <row r="9" ht="84" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>3</t>
@@ -1057,37 +1052,37 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Paseo del CBD de Futian</t>
+          <t>Centro Pokémon, 前海壹方城 Uniwalk, B2, 捣谷岛谷. 新湖路99号, Bao'an</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>El paseo es de día. Iluminación de las torres 19:00–22:00. Un jueves no pide reserva</t>
+          <t>Jueves 10:00–22:00. Viernes y sábado hasta las 22:30</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Gratis</t>
+          <t>Entrada gratis. Pagáis solo lo que compréis</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>No hace falta volver al hotel si venís de Lianhua: se baja andando. Desde el hotel, si vais solo a las torres: 20–25 min a pie hacia el norte, o taxi 10 min hasta 市民中心.</t>
+          <t>Desde el hotel: metro línea 1 dirección 机场东 hasta 宝安中心, salida F, 45–55 min, unos 7 ¥ por persona. Desde Lianhua, que es el caso: taxi 40–60 min, 80–140 ¥ (11–19 €). Texto: 请到宝安区新湖路99号前海壹方城，宝安中心地铁站F口</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>A pie 15–25 min si ya estáis en la parte baja, o línea 1 desde 购物公园 o 会展中心 hasta 岗厦.</t>
+          <t>Metro línea 1 dirección 罗湖 hasta 岗厦, unos 50 min. Taxi 40–70 min según el tráfico.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Seguid andando hasta CoCo Park (salida C de 购物公园).</t>
+          <t>Metro línea 1 dirección 罗湖, bajada en 购物公园. Os deja en CoCo Park.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>CBD</t>
+          <t>Uniwalk</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -1095,225 +1090,173 @@
           <t>Amap</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>CoCo Park 星河COCO Park</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>10:00–22:00, horario habitual del centro</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Entrada gratis</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Desde el hotel: línea 1 dirección 机场东, 2 paradas, 购物公园, salida C. Unos 10 min. Taxi 10 min, 15–25 ¥ (2–3 €).</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Línea 1 dirección 罗湖, 2 paradas, 岗厦, salida E.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Línea 1 dos paradas hasta 岗厦 y 10 min a pie a Harmay. Si saltáis Harmay, línea 10 una parada hasta Shuiwei.</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>CoCo Park</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Amap</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>Amap corto</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>CoCo Park 星河COCO Park</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>10:00–22:00, horario habitual del centro</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Entrada gratis</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Metro, mejor opción. Línea 1 en 岗厦, dirección 机场东, 2 paradas, 购物公园, salida C. Unos 10 min, unos 3 ¥ por persona. Taxi 10 min, 15–25 ¥ (2–3 €).</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Línea 1 dirección 罗湖, 2 paradas, 岗厦, salida E.</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Volved al hotel a descansar. Por la noche, Harmay y Riad están a 10 min a pie.</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>CoCo Park</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
+    <row r="11" ht="84" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Harmay, One Avenue 卓悦中心</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>10:00–22:00</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Entrada gratis. El precio depende del producto</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>A pie, 10 min hacia el norte (salida B de 岗厦). No está en UpperHills.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>A pie, 10 min.</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Línea 10 dirección 福田口岸, 1 parada, 福民, salida D.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Harmay</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>Amap</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>Amap corto</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Harmay, One Avenue 卓悦中心</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>10:00–22:00</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Entrada gratis. El precio depende del producto</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>A pie, 10 minutos hacia el norte (Gangxia salida B / Fuhua 1st Road). No hace falta taxi ni metro.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>A pie, 10 min.</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Riad está en el mismo centro. Seguid a pie.</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Harmay</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Shuiwei Night Market 水围夜市</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Desde las 16:00 hasta cerca de las 2:00</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Entrada gratis. Ración 15–40 ¥ (2–5 €). Cena para dos 80–150 ¥ (11–20 €)</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Metro. Línea 10 dirección 福田口岸, 1 parada, 福民, salida D, 5–8 min a pie. Unos 20 min, unos 2 ¥. Taxi 10 min, 15–25 ¥ (2–3 €).</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Línea 10 dirección 双拥街, 1 parada, 岗厦.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Fin del día.</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Shuiwei</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Amap</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>Amap corto</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="78" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Riad by The Theatre</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>The Theatre, en el mismo One Avenue, figura 14:00–02:00. Las torres, 19:00–22:00</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Sin entrada. Reservad terraza. Cóctel habitual en la zona 70–120 ¥ (9–16 €); no hay carta oficial publicada</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>A pie, los mismos 10 minutos que Harmay.</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>A pie, 10 min.</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Metro línea 10 dirección 福田口岸, 1 parada, 福民, salida D. O taxi 10 min hasta Shuiwei.</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Riad</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Amap</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Amap corto</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Shuiwei Night Market 水围夜市</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Puestos desde las 16:00 hasta cerca de las 2:00</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Entrada gratis. Ración 15–40 ¥ (2–5 €). Cena para dos 80–150 ¥ (11–20 €)</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Metro, mejor opción. Línea 10 en 岗厦, dirección 福田口岸, 1 parada, 福民, salida D, 5–8 min a pie. Unos 20 min, unos 2 ¥ por persona. Taxi 10 min, 15–25 ¥ (2–3 €).</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Línea 10 dirección 双拥街, 1 parada, 岗厦. O taxi.</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Fin del día. Vuelta al hotel.</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>Shuiwei</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>Amap</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>Amap corto</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:J13"/>
+  <autoFilter ref="A4:J12"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId1"/>
@@ -1329,24 +1272,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId22"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LDía 5 · 5 nov 2026 · Shenzhen Futian</oddHeader>
+    <oddHeader>&amp;LDía 5 · 5 nov 2026 · Shenzhen</oddHeader>
     <oddFooter>&amp;R1 € = 7,55 ¥ · 4 oct 2026</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1362,43 +1301,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Alternativas del día 5 — una sola, no las dos</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
+          <t>Luces: pasan al viernes 6. Alternativas: no caben hoy si hacéis el Pokémon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>El museo es gratis y cae en la bajada del CBD. Ping An es de pago y está al lado de CoCo Park; un jueves cierra a las 20:00. Después del vuelo nocturno no caben los dos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Noviembre: pases a las 19:00, 20:00 y 21:00. La plaza del Civic Center pide reserva gratis en el miniprograma 福田中心区夜景灯光预约导引服务. Riad está al lado, por si queréis ver las torres desde ahí. La tabla completa del viernes se hace cuando cerréis ese día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Opción</t>
+          <t>Qué</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Horario del jueves 5</t>
+          <t>Cuándo</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1413,140 +1351,215 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Dónde encaja en la ruta</t>
+          <t>Encaje</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Volver al hotel</t>
+          <t>Google Maps</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Amap</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
+          <t>Amap corto</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Espectáculo de luces del Civic Center</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Viernes 6 de noviembre. Pases 19:00, 20:00 y 21:00. Reserva para la plaza</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Gratis</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>A pie 20–25 min hacia el norte, o taxi 10 min hasta 市民中心.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>No es el jueves. Queda para el día 6.</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Civic Center</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
           <t>Amap</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Amap (enlace corto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="96" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Museo de Shenzhen, sala de historia y folklore, dentro del Civic Center</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Abierto (cierra los lunes). 10:00–18:00, última entrada 17:30. Pasaporte extranjero: carril verde, sin reserva</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Amap corto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Riad by The Theatre, One Avenue</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>El local figura 14:00–02:00. Útil el viernes, con las luces</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Sin entrada. Cóctel habitual 70–120 ¥ (9–16 €)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>A pie, 10 min desde el hotel.</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Opcional el viernes, al lado del CBD. No hace falta el jueves.</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Riad</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Amap</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Amap corto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Museo de Shenzhen, historia y folklore</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Jueves 10:00–18:00, última entrada 17:30. Pasaporte: carril verde</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Gratis</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Taxi 10 min hasta 市民中心, 15–25 ¥ (2–3 €). Metro: línea 1 una parada hasta 会展中心, transbordo a la línea 4 una parada hasta 市民中心. A pie 25 min hacia el norte.</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>En la bajada de Lianhua al CBD, si entráis antes de las 17:30. Calculad 60–90 min. Si entráis, acortad CoCo Park. No lo combinéis con Ping An.</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Línea 1 desde 会展中心 hasta 岗厦, salida E. O taxi 10 min.</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Taxi 10 min, 15–25 ¥. Metro: línea 1 a 会展中心 y línea 4 a 市民中心.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>No encaja hoy. La bajada de Lianhua va al taxi hacia Qianhai.</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Museo</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Amap</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="96" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Mirador Free Sky, planta 116 del Ping An Finance Center, 益田路5033号. Tel. 0755-29163888</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>10:00–20:00. Última entrada 19:15</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>180 ¥ por persona si se compra antes (24 €). El mismo día, 200 ¥ (26 €). Dos personas: 48–53 €</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>El mismo metro que CoCo Park: línea 1 hasta 购物公园, salida D, un minuto a pie. Taxi 10–15 min, 15–30 ¥ (2–4 €).</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>En el hueco de CoCo Park, entrando sobre las 16:30 para coger la luz de la tarde. Hora y media. Si subís, saltad el museo.</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Línea 1 desde 购物公园, dirección 罗湖, hasta 岗厦, salida E.</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Mirador Free Sky, Ping An, planta 116. Tel. 0755-29163888</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Jueves 10:00–20:00, última entrada 19:15</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>180 ¥ antes (24 €) o 200 ¥ el mismo día (26 €). Dos personas 48–53 €</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Línea 1 hasta 购物公园, salida D.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Solo si cambiáis la hora de CoCo Park por la subida y llegáis antes de las 18:00.</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Ping An</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Amap</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I6"/>
+  <autoFilter ref="A4:H8"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId10"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LDía 5 · 5 nov 2026 · Shenzhen Futian</oddHeader>
+    <oddHeader>&amp;LDía 5 · 5 nov 2026 · Shenzhen</oddHeader>
     <oddFooter>&amp;R1 € = 7,55 ¥ · 4 oct 2026</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>